<commit_message>
LMDI: Fjern MustSupport fra category i Legemiddeladministrering bfe6985cc24aeddd7bad4c6eaa4ff63f7ed55a1d
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-medicationadministration.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-medicationadministration.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2619" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2618" uniqueCount="480">
   <si>
     <t>Property</t>
   </si>
@@ -592,16 +592,13 @@
     <t>MedicationAdministration.category</t>
   </si>
   <si>
-    <t>Type of medication usage</t>
-  </si>
-  <si>
-    <t>Indicates where the medication is expected to be consumed or administered.</t>
-  </si>
-  <si>
-    <t>A coded concept describing where the medication administered is expected to occur.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/medication-admin-category|4.0.1</t>
+    <t>Kategori (inneliggende | poliklinisk | selvadministrert | utskrivelse)</t>
+  </si>
+  <si>
+    <t>Kategoriserer administreringskonteksten. Bruk 'community' for selvadministrering — pasienten tar legemidlet selv, men det er utdelt av institusjonen.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/medication-admin-category</t>
   </si>
   <si>
     <t>.inboundRelationship[typeCode=COMP].source[classCode=OBS, moodCode=EVN, code="type of medication usage"].value</t>
@@ -3693,11 +3690,9 @@
       <c r="X16" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="Y16" t="s" s="2">
+      <c r="Y16" s="2"/>
+      <c r="Z16" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="Z16" t="s" s="2">
-        <v>188</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>78</v>
@@ -3733,7 +3728,7 @@
         <v>78</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AM16" t="s" s="2">
         <v>78</v>
@@ -3747,10 +3742,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3773,16 +3768,16 @@
         <v>89</v>
       </c>
       <c r="K17" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="L17" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="L17" t="s" s="2">
+      <c r="M17" t="s" s="2">
         <v>192</v>
       </c>
-      <c r="M17" t="s" s="2">
+      <c r="N17" t="s" s="2">
         <v>193</v>
-      </c>
-      <c r="N17" t="s" s="2">
-        <v>194</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3832,7 +3827,7 @@
         <v>78</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>88</v>
@@ -3847,16 +3842,16 @@
         <v>100</v>
       </c>
       <c r="AK17" t="s" s="2">
+        <v>194</v>
+      </c>
+      <c r="AL17" t="s" s="2">
         <v>195</v>
       </c>
-      <c r="AL17" t="s" s="2">
+      <c r="AM17" t="s" s="2">
         <v>196</v>
       </c>
-      <c r="AM17" t="s" s="2">
+      <c r="AN17" t="s" s="2">
         <v>197</v>
-      </c>
-      <c r="AN17" t="s" s="2">
-        <v>198</v>
       </c>
       <c r="AO17" t="s" s="2">
         <v>78</v>
@@ -3864,10 +3859,10 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3890,13 +3885,13 @@
         <v>89</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="L18" t="s" s="2">
         <v>200</v>
       </c>
-      <c r="L18" t="s" s="2">
+      <c r="M18" t="s" s="2">
         <v>201</v>
-      </c>
-      <c r="M18" t="s" s="2">
-        <v>202</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3947,7 +3942,7 @@
         <v>78</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>88</v>
@@ -3962,16 +3957,16 @@
         <v>100</v>
       </c>
       <c r="AK18" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="AL18" t="s" s="2">
         <v>203</v>
       </c>
-      <c r="AL18" t="s" s="2">
+      <c r="AM18" t="s" s="2">
         <v>204</v>
       </c>
-      <c r="AM18" t="s" s="2">
+      <c r="AN18" t="s" s="2">
         <v>205</v>
-      </c>
-      <c r="AN18" t="s" s="2">
-        <v>206</v>
       </c>
       <c r="AO18" t="s" s="2">
         <v>78</v>
@@ -3979,10 +3974,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -4005,13 +4000,13 @@
         <v>78</v>
       </c>
       <c r="K19" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="L19" t="s" s="2">
         <v>208</v>
       </c>
-      <c r="L19" t="s" s="2">
+      <c r="M19" t="s" s="2">
         <v>209</v>
-      </c>
-      <c r="M19" t="s" s="2">
-        <v>210</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -4062,7 +4057,7 @@
         <v>78</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>79</v>
@@ -4077,16 +4072,16 @@
         <v>100</v>
       </c>
       <c r="AK19" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="AL19" t="s" s="2">
         <v>211</v>
       </c>
-      <c r="AL19" t="s" s="2">
+      <c r="AM19" t="s" s="2">
         <v>212</v>
       </c>
-      <c r="AM19" t="s" s="2">
+      <c r="AN19" t="s" s="2">
         <v>213</v>
-      </c>
-      <c r="AN19" t="s" s="2">
-        <v>214</v>
       </c>
       <c r="AO19" t="s" s="2">
         <v>78</v>
@@ -4094,10 +4089,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4120,13 +4115,13 @@
         <v>78</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>216</v>
       </c>
-      <c r="L20" t="s" s="2">
+      <c r="M20" t="s" s="2">
         <v>217</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>218</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -4177,7 +4172,7 @@
         <v>78</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -4195,10 +4190,10 @@
         <v>78</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AN20" t="s" s="2">
         <v>78</v>
@@ -4209,10 +4204,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -4235,13 +4230,13 @@
         <v>89</v>
       </c>
       <c r="K21" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="L21" t="s" s="2">
         <v>221</v>
       </c>
-      <c r="L21" t="s" s="2">
+      <c r="M21" t="s" s="2">
         <v>222</v>
-      </c>
-      <c r="M21" t="s" s="2">
-        <v>223</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -4280,17 +4275,17 @@
         <v>78</v>
       </c>
       <c r="AB21" t="s" s="2">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AC21" s="2"/>
       <c r="AD21" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE21" t="s" s="2">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>88</v>
@@ -4305,16 +4300,16 @@
         <v>100</v>
       </c>
       <c r="AK21" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="AL21" t="s" s="2">
         <v>226</v>
       </c>
-      <c r="AL21" t="s" s="2">
+      <c r="AM21" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AM21" t="s" s="2">
+      <c r="AN21" t="s" s="2">
         <v>228</v>
-      </c>
-      <c r="AN21" t="s" s="2">
-        <v>229</v>
       </c>
       <c r="AO21" t="s" s="2">
         <v>78</v>
@@ -4322,13 +4317,13 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
+        <v>229</v>
+      </c>
+      <c r="B22" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="C22" t="s" s="2">
         <v>230</v>
-      </c>
-      <c r="B22" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="C22" t="s" s="2">
-        <v>231</v>
       </c>
       <c r="D22" t="s" s="2">
         <v>78</v>
@@ -4350,13 +4345,13 @@
         <v>89</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>231</v>
+      </c>
+      <c r="L22" t="s" s="2">
         <v>232</v>
       </c>
-      <c r="L22" t="s" s="2">
-        <v>233</v>
-      </c>
       <c r="M22" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -4407,7 +4402,7 @@
         <v>78</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>88</v>
@@ -4419,19 +4414,19 @@
         <v>78</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AK22" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="AL22" t="s" s="2">
         <v>226</v>
       </c>
-      <c r="AL22" t="s" s="2">
+      <c r="AM22" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AM22" t="s" s="2">
+      <c r="AN22" t="s" s="2">
         <v>228</v>
-      </c>
-      <c r="AN22" t="s" s="2">
-        <v>229</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>78</v>
@@ -4439,13 +4434,13 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
+        <v>234</v>
+      </c>
+      <c r="B23" t="s" s="2">
+        <v>219</v>
+      </c>
+      <c r="C23" t="s" s="2">
         <v>235</v>
-      </c>
-      <c r="B23" t="s" s="2">
-        <v>220</v>
-      </c>
-      <c r="C23" t="s" s="2">
-        <v>236</v>
       </c>
       <c r="D23" t="s" s="2">
         <v>78</v>
@@ -4467,13 +4462,13 @@
         <v>89</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -4524,7 +4519,7 @@
         <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>88</v>
@@ -4539,16 +4534,16 @@
         <v>100</v>
       </c>
       <c r="AK23" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="AL23" t="s" s="2">
         <v>226</v>
       </c>
-      <c r="AL23" t="s" s="2">
+      <c r="AM23" t="s" s="2">
         <v>227</v>
       </c>
-      <c r="AM23" t="s" s="2">
+      <c r="AN23" t="s" s="2">
         <v>228</v>
-      </c>
-      <c r="AN23" t="s" s="2">
-        <v>229</v>
       </c>
       <c r="AO23" t="s" s="2">
         <v>78</v>
@@ -4556,10 +4551,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="B24" t="s" s="2">
         <v>238</v>
-      </c>
-      <c r="B24" t="s" s="2">
-        <v>239</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4582,13 +4577,13 @@
         <v>78</v>
       </c>
       <c r="K24" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L24" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="L24" t="s" s="2">
+      <c r="M24" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="M24" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4639,25 +4634,25 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="AG24" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH24" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI24" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ24" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK24" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL24" t="s" s="2">
         <v>243</v>
-      </c>
-      <c r="AG24" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH24" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI24" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ24" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK24" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL24" t="s" s="2">
-        <v>244</v>
       </c>
       <c r="AM24" t="s" s="2">
         <v>78</v>
@@ -4671,10 +4666,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
+        <v>244</v>
+      </c>
+      <c r="B25" t="s" s="2">
         <v>245</v>
-      </c>
-      <c r="B25" t="s" s="2">
-        <v>246</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4703,7 +4698,7 @@
         <v>135</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N25" t="s" s="2">
         <v>137</v>
@@ -4744,19 +4739,19 @@
         <v>78</v>
       </c>
       <c r="AB25" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="AC25" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="AC25" t="s" s="2">
+      <c r="AD25" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE25" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="AD25" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE25" t="s" s="2">
+      <c r="AF25" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="AF25" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -4774,7 +4769,7 @@
         <v>78</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>78</v>
@@ -4788,10 +4783,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="B26" t="s" s="2">
         <v>252</v>
-      </c>
-      <c r="B26" t="s" s="2">
-        <v>253</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4814,16 +4809,16 @@
         <v>89</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="L26" t="s" s="2">
+        <v>253</v>
+      </c>
+      <c r="M26" t="s" s="2">
         <v>254</v>
       </c>
-      <c r="M26" t="s" s="2">
+      <c r="N26" t="s" s="2">
         <v>255</v>
-      </c>
-      <c r="N26" t="s" s="2">
-        <v>256</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4873,31 +4868,31 @@
         <v>78</v>
       </c>
       <c r="AF26" t="s" s="2">
+        <v>256</v>
+      </c>
+      <c r="AG26" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH26" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI26" t="s" s="2">
         <v>257</v>
       </c>
-      <c r="AG26" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH26" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI26" t="s" s="2">
+      <c r="AJ26" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="AK26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL26" t="s" s="2">
         <v>258</v>
       </c>
-      <c r="AJ26" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="AK26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL26" t="s" s="2">
+      <c r="AM26" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN26" t="s" s="2">
         <v>259</v>
-      </c>
-      <c r="AM26" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN26" t="s" s="2">
-        <v>260</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>78</v>
@@ -4905,10 +4900,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="B27" t="s" s="2">
         <v>261</v>
-      </c>
-      <c r="B27" t="s" s="2">
-        <v>262</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4931,92 +4926,92 @@
         <v>89</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>262</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>263</v>
       </c>
-      <c r="M27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>264</v>
-      </c>
-      <c r="N27" t="s" s="2">
-        <v>265</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>78</v>
       </c>
       <c r="Q27" t="s" s="2">
+        <v>265</v>
+      </c>
+      <c r="R27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF27" t="s" s="2">
         <v>266</v>
       </c>
-      <c r="R27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF27" t="s" s="2">
+      <c r="AG27" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH27" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI27" t="s" s="2">
+        <v>257</v>
+      </c>
+      <c r="AJ27" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="AK27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL27" t="s" s="2">
         <v>267</v>
       </c>
-      <c r="AG27" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH27" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI27" t="s" s="2">
-        <v>258</v>
-      </c>
-      <c r="AJ27" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="AK27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL27" t="s" s="2">
+      <c r="AM27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN27" t="s" s="2">
         <v>268</v>
-      </c>
-      <c r="AM27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN27" t="s" s="2">
-        <v>269</v>
       </c>
       <c r="AO27" t="s" s="2">
         <v>78</v>
@@ -5024,10 +5019,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5050,13 +5045,13 @@
         <v>89</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>270</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>272</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>273</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -5107,7 +5102,7 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>79</v>
@@ -5122,16 +5117,16 @@
         <v>100</v>
       </c>
       <c r="AK28" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="AL28" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="AL28" t="s" s="2">
+      <c r="AM28" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="AM28" t="s" s="2">
+      <c r="AN28" t="s" s="2">
         <v>276</v>
-      </c>
-      <c r="AN28" t="s" s="2">
-        <v>277</v>
       </c>
       <c r="AO28" t="s" s="2">
         <v>78</v>
@@ -5139,10 +5134,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5165,13 +5160,13 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="L29" t="s" s="2">
+      <c r="M29" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -5222,25 +5217,25 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="AG29" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH29" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI29" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ29" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK29" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL29" t="s" s="2">
         <v>243</v>
-      </c>
-      <c r="AG29" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH29" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL29" t="s" s="2">
-        <v>244</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>78</v>
@@ -5254,10 +5249,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5286,7 +5281,7 @@
         <v>135</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N30" t="s" s="2">
         <v>137</v>
@@ -5339,7 +5334,7 @@
         <v>78</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
@@ -5357,7 +5352,7 @@
         <v>78</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>78</v>
@@ -5371,14 +5366,14 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5400,10 +5395,10 @@
         <v>134</v>
       </c>
       <c r="L31" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="M31" t="s" s="2">
         <v>282</v>
-      </c>
-      <c r="M31" t="s" s="2">
-        <v>283</v>
       </c>
       <c r="N31" t="s" s="2">
         <v>137</v>
@@ -5458,7 +5453,7 @@
         <v>78</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
@@ -5490,10 +5485,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5519,10 +5514,10 @@
         <v>175</v>
       </c>
       <c r="L32" t="s" s="2">
+        <v>285</v>
+      </c>
+      <c r="M32" t="s" s="2">
         <v>286</v>
-      </c>
-      <c r="M32" t="s" s="2">
-        <v>287</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5552,11 +5547,11 @@
         <v>178</v>
       </c>
       <c r="Y32" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="Z32" t="s" s="2">
         <v>288</v>
       </c>
-      <c r="Z32" t="s" s="2">
-        <v>289</v>
-      </c>
       <c r="AA32" t="s" s="2">
         <v>78</v>
       </c>
@@ -5573,7 +5568,7 @@
         <v>78</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -5588,10 +5583,10 @@
         <v>100</v>
       </c>
       <c r="AK32" t="s" s="2">
+        <v>289</v>
+      </c>
+      <c r="AL32" t="s" s="2">
         <v>290</v>
-      </c>
-      <c r="AL32" t="s" s="2">
-        <v>291</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>78</v>
@@ -5605,10 +5600,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5631,13 +5626,13 @@
         <v>89</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="L33" t="s" s="2">
         <v>293</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="M33" t="s" s="2">
         <v>294</v>
-      </c>
-      <c r="M33" t="s" s="2">
-        <v>295</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5688,7 +5683,7 @@
         <v>78</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>88</v>
@@ -5703,10 +5698,10 @@
         <v>100</v>
       </c>
       <c r="AK33" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="AL33" t="s" s="2">
         <v>296</v>
-      </c>
-      <c r="AL33" t="s" s="2">
-        <v>297</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>78</v>
@@ -5720,10 +5715,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5749,10 +5744,10 @@
         <v>175</v>
       </c>
       <c r="L34" t="s" s="2">
+        <v>298</v>
+      </c>
+      <c r="M34" t="s" s="2">
         <v>299</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>300</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5782,11 +5777,11 @@
         <v>178</v>
       </c>
       <c r="Y34" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="Z34" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="Z34" t="s" s="2">
-        <v>302</v>
-      </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
       </c>
@@ -5803,7 +5798,7 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5818,16 +5813,16 @@
         <v>100</v>
       </c>
       <c r="AK34" t="s" s="2">
+        <v>302</v>
+      </c>
+      <c r="AL34" t="s" s="2">
         <v>303</v>
       </c>
-      <c r="AL34" t="s" s="2">
+      <c r="AM34" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN34" t="s" s="2">
         <v>304</v>
-      </c>
-      <c r="AM34" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN34" t="s" s="2">
-        <v>305</v>
       </c>
       <c r="AO34" t="s" s="2">
         <v>78</v>
@@ -5835,10 +5830,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5861,16 +5856,16 @@
         <v>78</v>
       </c>
       <c r="K35" t="s" s="2">
+        <v>306</v>
+      </c>
+      <c r="L35" t="s" s="2">
         <v>307</v>
       </c>
-      <c r="L35" t="s" s="2">
+      <c r="M35" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="M35" t="s" s="2">
+      <c r="N35" t="s" s="2">
         <v>309</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>310</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -5920,7 +5915,7 @@
         <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5935,27 +5930,27 @@
         <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
+        <v>310</v>
+      </c>
+      <c r="AL35" t="s" s="2">
         <v>311</v>
       </c>
-      <c r="AL35" t="s" s="2">
+      <c r="AM35" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="AM35" t="s" s="2">
+      <c r="AN35" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO35" t="s" s="2">
         <v>313</v>
-      </c>
-      <c r="AN35" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AO35" t="s" s="2">
-        <v>314</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5978,16 +5973,16 @@
         <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="L36" t="s" s="2">
         <v>316</v>
       </c>
-      <c r="L36" t="s" s="2">
+      <c r="M36" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>318</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>319</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
@@ -6037,7 +6032,7 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -6052,16 +6047,16 @@
         <v>100</v>
       </c>
       <c r="AK36" t="s" s="2">
+        <v>319</v>
+      </c>
+      <c r="AL36" t="s" s="2">
         <v>320</v>
       </c>
-      <c r="AL36" t="s" s="2">
+      <c r="AM36" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN36" t="s" s="2">
         <v>321</v>
-      </c>
-      <c r="AM36" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN36" t="s" s="2">
-        <v>322</v>
       </c>
       <c r="AO36" t="s" s="2">
         <v>78</v>
@@ -6069,10 +6064,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6095,13 +6090,13 @@
         <v>78</v>
       </c>
       <c r="K37" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="L37" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="L37" t="s" s="2">
+      <c r="M37" t="s" s="2">
         <v>325</v>
-      </c>
-      <c r="M37" t="s" s="2">
-        <v>326</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -6152,7 +6147,7 @@
         <v>78</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
@@ -6170,13 +6165,13 @@
         <v>78</v>
       </c>
       <c r="AL37" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="AM37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN37" t="s" s="2">
         <v>327</v>
-      </c>
-      <c r="AM37" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN37" t="s" s="2">
-        <v>328</v>
       </c>
       <c r="AO37" t="s" s="2">
         <v>78</v>
@@ -6184,10 +6179,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6210,13 +6205,13 @@
         <v>78</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="L38" t="s" s="2">
         <v>330</v>
       </c>
-      <c r="L38" t="s" s="2">
+      <c r="M38" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="M38" t="s" s="2">
-        <v>332</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -6267,7 +6262,7 @@
         <v>78</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
@@ -6282,10 +6277,10 @@
         <v>100</v>
       </c>
       <c r="AK38" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="AL38" t="s" s="2">
         <v>333</v>
-      </c>
-      <c r="AL38" t="s" s="2">
-        <v>334</v>
       </c>
       <c r="AM38" t="s" s="2">
         <v>78</v>
@@ -6299,10 +6294,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6325,13 +6320,13 @@
         <v>78</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="L39" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="M39" t="s" s="2">
         <v>336</v>
-      </c>
-      <c r="M39" t="s" s="2">
-        <v>337</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6382,7 +6377,7 @@
         <v>78</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
@@ -6394,13 +6389,13 @@
         <v>78</v>
       </c>
       <c r="AJ39" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="AK39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL39" t="s" s="2">
         <v>338</v>
-      </c>
-      <c r="AK39" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL39" t="s" s="2">
-        <v>339</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>78</v>
@@ -6414,10 +6409,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6440,13 +6435,13 @@
         <v>78</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="M40" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6497,25 +6492,25 @@
         <v>78</v>
       </c>
       <c r="AF40" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="AG40" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH40" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL40" t="s" s="2">
         <v>243</v>
-      </c>
-      <c r="AG40" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH40" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI40" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ40" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK40" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL40" t="s" s="2">
-        <v>244</v>
       </c>
       <c r="AM40" t="s" s="2">
         <v>78</v>
@@ -6529,10 +6524,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6561,7 +6556,7 @@
         <v>135</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>137</v>
@@ -6614,7 +6609,7 @@
         <v>78</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>79</v>
@@ -6632,7 +6627,7 @@
         <v>78</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>78</v>
@@ -6646,14 +6641,14 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6675,10 +6670,10 @@
         <v>134</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>282</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>283</v>
       </c>
       <c r="N42" t="s" s="2">
         <v>137</v>
@@ -6733,7 +6728,7 @@
         <v>78</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>79</v>
@@ -6765,10 +6760,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6791,13 +6786,13 @@
         <v>78</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L43" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>344</v>
-      </c>
-      <c r="M43" t="s" s="2">
-        <v>345</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6848,7 +6843,7 @@
         <v>78</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>79</v>
@@ -6866,7 +6861,7 @@
         <v>78</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>78</v>
@@ -6880,10 +6875,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6909,13 +6904,13 @@
         <v>175</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>348</v>
       </c>
-      <c r="M44" t="s" s="2">
+      <c r="N44" t="s" s="2">
         <v>349</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>350</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -6944,11 +6939,11 @@
         <v>178</v>
       </c>
       <c r="Y44" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="Z44" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="Z44" t="s" s="2">
-        <v>352</v>
-      </c>
       <c r="AA44" t="s" s="2">
         <v>78</v>
       </c>
@@ -6965,7 +6960,7 @@
         <v>78</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>79</v>
@@ -6983,13 +6978,13 @@
         <v>78</v>
       </c>
       <c r="AL44" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN44" t="s" s="2">
         <v>353</v>
-      </c>
-      <c r="AM44" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN44" t="s" s="2">
-        <v>354</v>
       </c>
       <c r="AO44" t="s" s="2">
         <v>78</v>
@@ -6997,10 +6992,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -7026,13 +7021,13 @@
         <v>175</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>356</v>
       </c>
-      <c r="M45" t="s" s="2">
+      <c r="N45" t="s" s="2">
         <v>357</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>358</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -7061,11 +7056,11 @@
         <v>178</v>
       </c>
       <c r="Y45" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="Z45" t="s" s="2">
         <v>359</v>
       </c>
-      <c r="Z45" t="s" s="2">
-        <v>360</v>
-      </c>
       <c r="AA45" t="s" s="2">
         <v>78</v>
       </c>
@@ -7082,7 +7077,7 @@
         <v>78</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
@@ -7100,13 +7095,13 @@
         <v>78</v>
       </c>
       <c r="AL45" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN45" t="s" s="2">
         <v>361</v>
-      </c>
-      <c r="AM45" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN45" t="s" s="2">
-        <v>362</v>
       </c>
       <c r="AO45" t="s" s="2">
         <v>78</v>
@@ -7114,10 +7109,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7140,13 +7135,13 @@
         <v>78</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7197,25 +7192,25 @@
         <v>78</v>
       </c>
       <c r="AF46" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL46" t="s" s="2">
         <v>243</v>
-      </c>
-      <c r="AG46" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH46" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI46" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ46" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK46" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL46" t="s" s="2">
-        <v>244</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>78</v>
@@ -7229,10 +7224,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7261,7 +7256,7 @@
         <v>135</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N47" t="s" s="2">
         <v>137</v>
@@ -7302,19 +7297,19 @@
         <v>78</v>
       </c>
       <c r="AB47" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="AC47" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="AC47" t="s" s="2">
+      <c r="AD47" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE47" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="AD47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE47" t="s" s="2">
+      <c r="AF47" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="AF47" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>79</v>
@@ -7332,7 +7327,7 @@
         <v>78</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM47" t="s" s="2">
         <v>78</v>
@@ -7346,10 +7341,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7372,19 +7367,19 @@
         <v>89</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>367</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>368</v>
       </c>
-      <c r="N48" t="s" s="2">
+      <c r="O48" t="s" s="2">
         <v>369</v>
-      </c>
-      <c r="O48" t="s" s="2">
-        <v>370</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>78</v>
@@ -7421,17 +7416,17 @@
         <v>78</v>
       </c>
       <c r="AB48" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AC48" s="2"/>
       <c r="AD48" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE48" t="s" s="2">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>79</v>
@@ -7449,13 +7444,13 @@
         <v>78</v>
       </c>
       <c r="AL48" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="AM48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN48" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="AM48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="AO48" t="s" s="2">
         <v>78</v>
@@ -7463,13 +7458,13 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="C49" t="s" s="2">
         <v>375</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>365</v>
-      </c>
-      <c r="C49" t="s" s="2">
-        <v>376</v>
       </c>
       <c r="D49" t="s" s="2">
         <v>78</v>
@@ -7491,19 +7486,19 @@
         <v>89</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="L49" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>377</v>
       </c>
-      <c r="M49" t="s" s="2">
-        <v>378</v>
-      </c>
       <c r="N49" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="O49" t="s" s="2">
         <v>369</v>
-      </c>
-      <c r="O49" t="s" s="2">
-        <v>370</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>78</v>
@@ -7552,7 +7547,7 @@
         <v>78</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>79</v>
@@ -7570,13 +7565,13 @@
         <v>78</v>
       </c>
       <c r="AL49" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN49" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="AO49" t="s" s="2">
         <v>78</v>
@@ -7584,10 +7579,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="B50" t="s" s="2">
         <v>379</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>380</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7610,13 +7605,13 @@
         <v>78</v>
       </c>
       <c r="K50" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L50" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="L50" t="s" s="2">
+      <c r="M50" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7667,25 +7662,25 @@
         <v>78</v>
       </c>
       <c r="AF50" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL50" t="s" s="2">
         <v>243</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>244</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>78</v>
@@ -7699,10 +7694,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
+        <v>380</v>
+      </c>
+      <c r="B51" t="s" s="2">
         <v>381</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>382</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7731,7 +7726,7 @@
         <v>135</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N51" t="s" s="2">
         <v>137</v>
@@ -7772,19 +7767,19 @@
         <v>78</v>
       </c>
       <c r="AB51" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="AC51" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="AC51" t="s" s="2">
+      <c r="AD51" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE51" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="AD51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE51" t="s" s="2">
+      <c r="AF51" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>79</v>
@@ -7802,7 +7797,7 @@
         <v>78</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM51" t="s" s="2">
         <v>78</v>
@@ -7816,10 +7811,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="B52" t="s" s="2">
         <v>383</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>384</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7845,16 +7840,16 @@
         <v>102</v>
       </c>
       <c r="L52" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="M52" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="M52" t="s" s="2">
+      <c r="N52" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="N52" t="s" s="2">
+      <c r="O52" t="s" s="2">
         <v>387</v>
-      </c>
-      <c r="O52" t="s" s="2">
-        <v>388</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>78</v>
@@ -7864,46 +7859,46 @@
         <v>78</v>
       </c>
       <c r="S52" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="T52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF52" t="s" s="2">
         <v>389</v>
-      </c>
-      <c r="T52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF52" t="s" s="2">
-        <v>390</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>79</v>
@@ -7921,13 +7916,13 @@
         <v>78</v>
       </c>
       <c r="AL52" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="AM52" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN52" t="s" s="2">
         <v>391</v>
-      </c>
-      <c r="AM52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>392</v>
       </c>
       <c r="AO52" t="s" s="2">
         <v>78</v>
@@ -7935,10 +7930,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
+        <v>392</v>
+      </c>
+      <c r="B53" t="s" s="2">
         <v>393</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>394</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7961,16 +7956,16 @@
         <v>89</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="M53" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="M53" t="s" s="2">
+      <c r="N53" t="s" s="2">
         <v>396</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>397</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -8020,7 +8015,7 @@
         <v>78</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>79</v>
@@ -8038,13 +8033,13 @@
         <v>78</v>
       </c>
       <c r="AL53" t="s" s="2">
+        <v>398</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN53" t="s" s="2">
         <v>399</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>400</v>
       </c>
       <c r="AO53" t="s" s="2">
         <v>78</v>
@@ -8052,10 +8047,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="B54" t="s" s="2">
         <v>401</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>402</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8081,14 +8076,14 @@
         <v>108</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>402</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>403</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>404</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" t="s" s="2">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>78</v>
@@ -8117,25 +8112,25 @@
       </c>
       <c r="Y54" s="2"/>
       <c r="Z54" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="AA54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF54" t="s" s="2">
         <v>406</v>
-      </c>
-      <c r="AA54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF54" t="s" s="2">
-        <v>407</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>79</v>
@@ -8153,13 +8148,13 @@
         <v>78</v>
       </c>
       <c r="AL54" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN54" t="s" s="2">
         <v>408</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>409</v>
       </c>
       <c r="AO54" t="s" s="2">
         <v>78</v>
@@ -8167,10 +8162,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="B55" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8193,17 +8188,17 @@
         <v>89</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L55" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>412</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>413</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>78</v>
@@ -8252,7 +8247,7 @@
         <v>78</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>79</v>
@@ -8270,13 +8265,13 @@
         <v>78</v>
       </c>
       <c r="AL55" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="AM55" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN55" t="s" s="2">
         <v>416</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>417</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>78</v>
@@ -8284,10 +8279,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="B56" t="s" s="2">
         <v>418</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>419</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8310,19 +8305,19 @@
         <v>89</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="L56" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="L56" t="s" s="2">
+      <c r="M56" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="M56" t="s" s="2">
+      <c r="N56" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="N56" t="s" s="2">
+      <c r="O56" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="O56" t="s" s="2">
-        <v>424</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>78</v>
@@ -8371,7 +8366,7 @@
         <v>78</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
@@ -8389,13 +8384,13 @@
         <v>78</v>
       </c>
       <c r="AL56" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="AM56" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN56" t="s" s="2">
         <v>426</v>
-      </c>
-      <c r="AM56" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN56" t="s" s="2">
-        <v>427</v>
       </c>
       <c r="AO56" t="s" s="2">
         <v>78</v>
@@ -8403,13 +8398,13 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="C57" t="s" s="2">
         <v>428</v>
-      </c>
-      <c r="B57" t="s" s="2">
-        <v>365</v>
-      </c>
-      <c r="C57" t="s" s="2">
-        <v>429</v>
       </c>
       <c r="D57" t="s" s="2">
         <v>78</v>
@@ -8431,19 +8426,19 @@
         <v>89</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="L57" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="M57" t="s" s="2">
         <v>430</v>
       </c>
-      <c r="M57" t="s" s="2">
-        <v>431</v>
-      </c>
       <c r="N57" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="O57" t="s" s="2">
         <v>369</v>
-      </c>
-      <c r="O57" t="s" s="2">
-        <v>370</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>78</v>
@@ -8492,7 +8487,7 @@
         <v>78</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>79</v>
@@ -8510,13 +8505,13 @@
         <v>78</v>
       </c>
       <c r="AL57" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN57" t="s" s="2">
         <v>373</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN57" t="s" s="2">
-        <v>374</v>
       </c>
       <c r="AO57" t="s" s="2">
         <v>78</v>
@@ -8524,10 +8519,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8550,13 +8545,13 @@
         <v>78</v>
       </c>
       <c r="K58" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="L58" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="L58" t="s" s="2">
+      <c r="M58" t="s" s="2">
         <v>241</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>242</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8607,25 +8602,25 @@
         <v>78</v>
       </c>
       <c r="AF58" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL58" t="s" s="2">
         <v>243</v>
-      </c>
-      <c r="AG58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH58" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI58" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ58" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AK58" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>244</v>
       </c>
       <c r="AM58" t="s" s="2">
         <v>78</v>
@@ -8639,10 +8634,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8671,7 +8666,7 @@
         <v>135</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="N59" t="s" s="2">
         <v>137</v>
@@ -8712,19 +8707,19 @@
         <v>78</v>
       </c>
       <c r="AB59" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="AC59" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="AC59" t="s" s="2">
+      <c r="AD59" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE59" t="s" s="2">
         <v>249</v>
       </c>
-      <c r="AD59" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE59" t="s" s="2">
+      <c r="AF59" t="s" s="2">
         <v>250</v>
-      </c>
-      <c r="AF59" t="s" s="2">
-        <v>251</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>79</v>
@@ -8742,7 +8737,7 @@
         <v>78</v>
       </c>
       <c r="AL59" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM59" t="s" s="2">
         <v>78</v>
@@ -8756,10 +8751,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8785,16 +8780,16 @@
         <v>102</v>
       </c>
       <c r="L60" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="M60" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="M60" t="s" s="2">
+      <c r="N60" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="N60" t="s" s="2">
+      <c r="O60" t="s" s="2">
         <v>387</v>
-      </c>
-      <c r="O60" t="s" s="2">
-        <v>388</v>
       </c>
       <c r="P60" t="s" s="2">
         <v>78</v>
@@ -8804,7 +8799,7 @@
         <v>78</v>
       </c>
       <c r="S60" t="s" s="2">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="T60" t="s" s="2">
         <v>78</v>
@@ -8843,7 +8838,7 @@
         <v>78</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>79</v>
@@ -8861,13 +8856,13 @@
         <v>78</v>
       </c>
       <c r="AL60" t="s" s="2">
+        <v>390</v>
+      </c>
+      <c r="AM60" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN60" t="s" s="2">
         <v>391</v>
-      </c>
-      <c r="AM60" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN60" t="s" s="2">
-        <v>392</v>
       </c>
       <c r="AO60" t="s" s="2">
         <v>78</v>
@@ -8875,10 +8870,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8901,16 +8896,16 @@
         <v>89</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L61" t="s" s="2">
+        <v>394</v>
+      </c>
+      <c r="M61" t="s" s="2">
         <v>395</v>
       </c>
-      <c r="M61" t="s" s="2">
+      <c r="N61" t="s" s="2">
         <v>396</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>397</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -8960,7 +8955,7 @@
         <v>78</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>79</v>
@@ -8978,13 +8973,13 @@
         <v>78</v>
       </c>
       <c r="AL61" t="s" s="2">
+        <v>398</v>
+      </c>
+      <c r="AM61" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN61" t="s" s="2">
         <v>399</v>
-      </c>
-      <c r="AM61" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>400</v>
       </c>
       <c r="AO61" t="s" s="2">
         <v>78</v>
@@ -8992,10 +8987,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9021,14 +9016,14 @@
         <v>108</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" t="s" s="2">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="P62" t="s" s="2">
         <v>78</v>
@@ -9077,7 +9072,7 @@
         <v>78</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>79</v>
@@ -9095,13 +9090,13 @@
         <v>78</v>
       </c>
       <c r="AL62" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="AM62" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN62" t="s" s="2">
         <v>408</v>
-      </c>
-      <c r="AM62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN62" t="s" s="2">
-        <v>409</v>
       </c>
       <c r="AO62" t="s" s="2">
         <v>78</v>
@@ -9109,10 +9104,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9135,17 +9130,17 @@
         <v>89</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>78</v>
@@ -9194,7 +9189,7 @@
         <v>78</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>79</v>
@@ -9212,13 +9207,13 @@
         <v>78</v>
       </c>
       <c r="AL63" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="AM63" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN63" t="s" s="2">
         <v>416</v>
-      </c>
-      <c r="AM63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN63" t="s" s="2">
-        <v>417</v>
       </c>
       <c r="AO63" t="s" s="2">
         <v>78</v>
@@ -9226,10 +9221,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9252,19 +9247,19 @@
         <v>89</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>420</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="M64" t="s" s="2">
+      <c r="N64" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="N64" t="s" s="2">
+      <c r="O64" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="O64" t="s" s="2">
-        <v>424</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>78</v>
@@ -9313,7 +9308,7 @@
         <v>78</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>79</v>
@@ -9331,13 +9326,13 @@
         <v>78</v>
       </c>
       <c r="AL64" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="AM64" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN64" t="s" s="2">
         <v>426</v>
-      </c>
-      <c r="AM64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN64" t="s" s="2">
-        <v>427</v>
       </c>
       <c r="AO64" t="s" s="2">
         <v>78</v>
@@ -9345,10 +9340,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9371,19 +9366,19 @@
         <v>89</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L65" t="s" s="2">
+        <v>442</v>
+      </c>
+      <c r="M65" t="s" s="2">
         <v>443</v>
       </c>
-      <c r="M65" t="s" s="2">
+      <c r="N65" t="s" s="2">
         <v>444</v>
       </c>
-      <c r="N65" t="s" s="2">
+      <c r="O65" t="s" s="2">
         <v>445</v>
-      </c>
-      <c r="O65" t="s" s="2">
-        <v>446</v>
       </c>
       <c r="P65" t="s" s="2">
         <v>78</v>
@@ -9432,7 +9427,7 @@
         <v>78</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>79</v>
@@ -9450,13 +9445,13 @@
         <v>78</v>
       </c>
       <c r="AL65" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="AM65" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN65" t="s" s="2">
         <v>448</v>
-      </c>
-      <c r="AM65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN65" t="s" s="2">
-        <v>449</v>
       </c>
       <c r="AO65" t="s" s="2">
         <v>78</v>
@@ -9464,10 +9459,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -9493,13 +9488,13 @@
         <v>175</v>
       </c>
       <c r="L66" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="M66" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="M66" t="s" s="2">
+      <c r="N66" t="s" s="2">
         <v>452</v>
-      </c>
-      <c r="N66" t="s" s="2">
-        <v>453</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
@@ -9528,11 +9523,11 @@
         <v>178</v>
       </c>
       <c r="Y66" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="Z66" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="Z66" t="s" s="2">
-        <v>455</v>
-      </c>
       <c r="AA66" t="s" s="2">
         <v>78</v>
       </c>
@@ -9549,7 +9544,7 @@
         <v>78</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>79</v>
@@ -9567,13 +9562,13 @@
         <v>78</v>
       </c>
       <c r="AL66" t="s" s="2">
+        <v>455</v>
+      </c>
+      <c r="AM66" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN66" t="s" s="2">
         <v>456</v>
-      </c>
-      <c r="AM66" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN66" t="s" s="2">
-        <v>457</v>
       </c>
       <c r="AO66" t="s" s="2">
         <v>78</v>
@@ -9581,10 +9576,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9607,16 +9602,16 @@
         <v>78</v>
       </c>
       <c r="K67" t="s" s="2">
+        <v>458</v>
+      </c>
+      <c r="L67" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="L67" t="s" s="2">
+      <c r="M67" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="M67" t="s" s="2">
+      <c r="N67" t="s" s="2">
         <v>461</v>
-      </c>
-      <c r="N67" t="s" s="2">
-        <v>462</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -9666,7 +9661,7 @@
         <v>78</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>79</v>
@@ -9684,13 +9679,13 @@
         <v>78</v>
       </c>
       <c r="AL67" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="AM67" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN67" t="s" s="2">
         <v>463</v>
-      </c>
-      <c r="AM67" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN67" t="s" s="2">
-        <v>464</v>
       </c>
       <c r="AO67" t="s" s="2">
         <v>78</v>
@@ -9698,10 +9693,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9724,16 +9719,16 @@
         <v>78</v>
       </c>
       <c r="K68" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="L68" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="L68" t="s" s="2">
+      <c r="M68" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>468</v>
-      </c>
-      <c r="N68" t="s" s="2">
-        <v>469</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
@@ -9771,17 +9766,17 @@
         <v>78</v>
       </c>
       <c r="AB68" t="s" s="2">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AC68" s="2"/>
       <c r="AD68" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE68" t="s" s="2">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>79</v>
@@ -9799,13 +9794,13 @@
         <v>78</v>
       </c>
       <c r="AL68" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AM68" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN68" t="s" s="2">
         <v>470</v>
-      </c>
-      <c r="AM68" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN68" t="s" s="2">
-        <v>471</v>
       </c>
       <c r="AO68" t="s" s="2">
         <v>78</v>
@@ -9813,13 +9808,13 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="B69" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="C69" t="s" s="2">
         <v>472</v>
-      </c>
-      <c r="B69" t="s" s="2">
-        <v>465</v>
-      </c>
-      <c r="C69" t="s" s="2">
-        <v>473</v>
       </c>
       <c r="D69" t="s" s="2">
         <v>78</v>
@@ -9841,16 +9836,16 @@
         <v>78</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="M69" t="s" s="2">
+      <c r="N69" t="s" s="2">
         <v>468</v>
-      </c>
-      <c r="N69" t="s" s="2">
-        <v>469</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -9900,7 +9895,7 @@
         <v>78</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>79</v>
@@ -9918,13 +9913,13 @@
         <v>78</v>
       </c>
       <c r="AL69" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AM69" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN69" t="s" s="2">
         <v>470</v>
-      </c>
-      <c r="AM69" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN69" t="s" s="2">
-        <v>471</v>
       </c>
       <c r="AO69" t="s" s="2">
         <v>78</v>
@@ -9932,10 +9927,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -9958,16 +9953,16 @@
         <v>78</v>
       </c>
       <c r="K70" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="L70" t="s" s="2">
         <v>476</v>
       </c>
-      <c r="L70" t="s" s="2">
+      <c r="M70" t="s" s="2">
         <v>477</v>
       </c>
-      <c r="M70" t="s" s="2">
+      <c r="N70" t="s" s="2">
         <v>478</v>
-      </c>
-      <c r="N70" t="s" s="2">
-        <v>479</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
@@ -10017,7 +10012,7 @@
         <v>78</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>79</v>
@@ -10035,7 +10030,7 @@
         <v>78</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>78</v>

</xml_diff>